<commit_message>
chore: sync GST statistics files 2026-10-01
</commit_message>
<xml_diff>
--- a/gstdatabase/GSTR-1-2017-2018.xlsx
+++ b/gstdatabase/GSTR-1-2017-2018.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GSTN\Krishnan Sir\Monthly Report\Jul-26\GST Statistics Downloads 31st Jul 26\Downloads\GSTR 1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GSTN\Krishnan Sir\Monthly Report\Aug-26\GST Statistics Downloads 31st Aug 26\Downloads\GSTR 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF840D9D-3AB6-4DA6-8FC4-6D525B75DBD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B278C8-BBA5-4735-94B1-5CC87F561424}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -182,10 +182,10 @@
     <t>Andaman and Nicobar Islands</t>
   </si>
   <si>
-    <t>Data Considered upto 31st Jul 2026</t>
+    <t>Data Considered upto 31st Aug 2026</t>
   </si>
   <si>
-    <t>Filing %age as on 31st Jul 2026</t>
+    <t>Filing %age as on 31st Aug 2026</t>
   </si>
 </sst>
 </file>
@@ -374,6 +374,15 @@
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="17" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -387,15 +396,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="17" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -736,10 +736,10 @@
       <c r="L2" s="8"/>
     </row>
     <row r="3" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="29"/>
+      <c r="B3" s="24"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -766,86 +766,86 @@
       <c r="L4" s="8"/>
     </row>
     <row r="5" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="29" t="s">
+      <c r="A5" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="29"/>
-      <c r="C5" s="29"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
     </row>
     <row r="7" spans="1:48" s="17" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="30" t="s">
+      <c r="A7" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="27">
         <v>42917</v>
       </c>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="28">
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="31">
         <v>42948</v>
       </c>
-      <c r="I7" s="28"/>
-      <c r="J7" s="28"/>
-      <c r="K7" s="28"/>
-      <c r="L7" s="28"/>
-      <c r="M7" s="24">
+      <c r="I7" s="31"/>
+      <c r="J7" s="31"/>
+      <c r="K7" s="31"/>
+      <c r="L7" s="31"/>
+      <c r="M7" s="27">
         <v>42979</v>
       </c>
-      <c r="N7" s="25"/>
-      <c r="O7" s="25"/>
-      <c r="P7" s="25"/>
-      <c r="Q7" s="25"/>
-      <c r="R7" s="28">
+      <c r="N7" s="28"/>
+      <c r="O7" s="28"/>
+      <c r="P7" s="28"/>
+      <c r="Q7" s="28"/>
+      <c r="R7" s="31">
         <v>43009</v>
       </c>
-      <c r="S7" s="28"/>
-      <c r="T7" s="28"/>
-      <c r="U7" s="28"/>
-      <c r="V7" s="28"/>
-      <c r="W7" s="24">
+      <c r="S7" s="31"/>
+      <c r="T7" s="31"/>
+      <c r="U7" s="31"/>
+      <c r="V7" s="31"/>
+      <c r="W7" s="27">
         <v>43040</v>
       </c>
-      <c r="X7" s="25"/>
-      <c r="Y7" s="25"/>
-      <c r="Z7" s="25"/>
-      <c r="AA7" s="25"/>
-      <c r="AB7" s="28">
+      <c r="X7" s="28"/>
+      <c r="Y7" s="28"/>
+      <c r="Z7" s="28"/>
+      <c r="AA7" s="28"/>
+      <c r="AB7" s="31">
         <v>43070</v>
       </c>
-      <c r="AC7" s="28"/>
-      <c r="AD7" s="28"/>
-      <c r="AE7" s="28"/>
-      <c r="AF7" s="28"/>
-      <c r="AG7" s="24">
+      <c r="AC7" s="31"/>
+      <c r="AD7" s="31"/>
+      <c r="AE7" s="31"/>
+      <c r="AF7" s="31"/>
+      <c r="AG7" s="27">
         <v>43101</v>
       </c>
-      <c r="AH7" s="25"/>
-      <c r="AI7" s="25"/>
-      <c r="AJ7" s="25"/>
-      <c r="AK7" s="25"/>
-      <c r="AL7" s="28">
+      <c r="AH7" s="28"/>
+      <c r="AI7" s="28"/>
+      <c r="AJ7" s="28"/>
+      <c r="AK7" s="28"/>
+      <c r="AL7" s="31">
         <v>43132</v>
       </c>
-      <c r="AM7" s="28"/>
-      <c r="AN7" s="28"/>
-      <c r="AO7" s="28"/>
-      <c r="AP7" s="28"/>
-      <c r="AQ7" s="24">
+      <c r="AM7" s="31"/>
+      <c r="AN7" s="31"/>
+      <c r="AO7" s="31"/>
+      <c r="AP7" s="31"/>
+      <c r="AQ7" s="27">
         <v>43160</v>
       </c>
-      <c r="AR7" s="25"/>
-      <c r="AS7" s="25"/>
-      <c r="AT7" s="25"/>
-      <c r="AU7" s="25"/>
+      <c r="AR7" s="28"/>
+      <c r="AS7" s="28"/>
+      <c r="AT7" s="28"/>
+      <c r="AU7" s="28"/>
     </row>
     <row r="8" spans="1:48" s="17" customFormat="1" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="30"/>
-      <c r="B8" s="31"/>
+      <c r="A8" s="25"/>
+      <c r="B8" s="26"/>
       <c r="C8" s="18" t="s">
         <v>4</v>
       </c>
@@ -1676,14 +1676,14 @@
       </c>
       <c r="O13" s="9">
         <f t="shared" si="4"/>
-        <v>21064</v>
+        <v>21066</v>
       </c>
       <c r="P13" s="22">
-        <v>87514</v>
+        <v>87516</v>
       </c>
       <c r="Q13" s="10">
         <f t="shared" si="5"/>
-        <v>0.8744579228202003</v>
+        <v>0.87447790723235874</v>
       </c>
       <c r="R13" s="6">
         <v>34094</v>
@@ -1727,14 +1727,14 @@
       </c>
       <c r="AD13" s="9">
         <f t="shared" si="10"/>
-        <v>22133</v>
+        <v>22135</v>
       </c>
       <c r="AE13" s="22">
-        <v>87330</v>
+        <v>87332</v>
       </c>
       <c r="AF13" s="10">
         <f t="shared" si="11"/>
-        <v>0.87543606399615059</v>
+        <v>0.87545611291551384</v>
       </c>
       <c r="AG13" s="6">
         <v>35615</v>
@@ -1778,14 +1778,14 @@
       </c>
       <c r="AS13" s="9">
         <f t="shared" si="16"/>
-        <v>28034</v>
+        <v>28038</v>
       </c>
       <c r="AT13" s="22">
-        <v>92883</v>
+        <v>92887</v>
       </c>
       <c r="AU13" s="10">
         <f t="shared" si="17"/>
-        <v>0.86325699840142756</v>
+        <v>0.86329417450462842</v>
       </c>
     </row>
     <row r="14" spans="1:48" x14ac:dyDescent="0.3">
@@ -2066,14 +2066,14 @@
       </c>
       <c r="AI15" s="9">
         <f t="shared" si="12"/>
-        <v>12379</v>
+        <v>12380</v>
       </c>
       <c r="AJ15" s="22">
-        <v>150147</v>
+        <v>150148</v>
       </c>
       <c r="AK15" s="10">
         <f t="shared" si="13"/>
-        <v>0.86595958197799161</v>
+        <v>0.86596534938980785</v>
       </c>
       <c r="AL15" s="6">
         <v>176069</v>
@@ -2159,14 +2159,14 @@
       </c>
       <c r="O16" s="9">
         <f t="shared" si="4"/>
-        <v>77979</v>
+        <v>77980</v>
       </c>
       <c r="P16" s="22">
-        <v>411133</v>
+        <v>411134</v>
       </c>
       <c r="Q16" s="10">
         <f t="shared" si="5"/>
-        <v>0.94311917766425268</v>
+        <v>0.94312147161579063</v>
       </c>
       <c r="R16" s="6">
         <v>119115</v>
@@ -2176,14 +2176,14 @@
       </c>
       <c r="T16" s="9">
         <f t="shared" si="6"/>
-        <v>6369</v>
+        <v>6370</v>
       </c>
       <c r="U16" s="22">
-        <v>105084</v>
+        <v>105085</v>
       </c>
       <c r="V16" s="10">
         <f t="shared" si="7"/>
-        <v>0.88220627125047224</v>
+        <v>0.88221466649876168</v>
       </c>
       <c r="W16" s="6">
         <v>119566</v>
@@ -2193,14 +2193,14 @@
       </c>
       <c r="Y16" s="9">
         <f t="shared" si="8"/>
-        <v>7876</v>
+        <v>7877</v>
       </c>
       <c r="Z16" s="22">
-        <v>107162</v>
+        <v>107163</v>
       </c>
       <c r="AA16" s="10">
         <f t="shared" si="9"/>
-        <v>0.89625813358312567</v>
+        <v>0.89626649716474582</v>
       </c>
       <c r="AB16" s="6">
         <v>433360</v>
@@ -2210,14 +2210,14 @@
       </c>
       <c r="AD16" s="9">
         <f t="shared" si="10"/>
-        <v>79141</v>
+        <v>79142</v>
       </c>
       <c r="AE16" s="22">
-        <v>412177</v>
+        <v>412178</v>
       </c>
       <c r="AF16" s="10">
         <f t="shared" si="11"/>
-        <v>0.95111916189772938</v>
+        <v>0.951121469448034</v>
       </c>
       <c r="AG16" s="6">
         <v>121543</v>
@@ -2227,14 +2227,14 @@
       </c>
       <c r="AI16" s="9">
         <f t="shared" si="12"/>
-        <v>8642</v>
+        <v>8643</v>
       </c>
       <c r="AJ16" s="22">
-        <v>107469</v>
+        <v>107470</v>
       </c>
       <c r="AK16" s="10">
         <f t="shared" si="13"/>
-        <v>0.88420558979126729</v>
+        <v>0.88421381733213755</v>
       </c>
       <c r="AL16" s="6">
         <v>122081</v>
@@ -2244,14 +2244,14 @@
       </c>
       <c r="AN16" s="9">
         <f t="shared" si="14"/>
-        <v>9229</v>
+        <v>9230</v>
       </c>
       <c r="AO16" s="22">
-        <v>107667</v>
+        <v>107668</v>
       </c>
       <c r="AP16" s="10">
         <f t="shared" si="15"/>
-        <v>0.88193084919029174</v>
+        <v>0.88193904047312854</v>
       </c>
       <c r="AQ16" s="6">
         <v>455889</v>
@@ -2261,14 +2261,14 @@
       </c>
       <c r="AS16" s="9">
         <f t="shared" si="16"/>
-        <v>94226</v>
+        <v>94231</v>
       </c>
       <c r="AT16" s="22">
-        <v>430121</v>
+        <v>430126</v>
       </c>
       <c r="AU16" s="10">
         <f t="shared" si="17"/>
-        <v>0.94347746929625409</v>
+        <v>0.94348843687827522</v>
       </c>
     </row>
     <row r="17" spans="1:47" x14ac:dyDescent="0.3">
@@ -2320,14 +2320,14 @@
       </c>
       <c r="O17" s="9">
         <f t="shared" si="4"/>
-        <v>168609</v>
+        <v>168610</v>
       </c>
       <c r="P17" s="22">
-        <v>800817</v>
+        <v>800818</v>
       </c>
       <c r="Q17" s="10">
         <f t="shared" si="5"/>
-        <v>0.90196721089906473</v>
+        <v>0.90196833720783554</v>
       </c>
       <c r="R17" s="6">
         <v>272330</v>
@@ -2371,14 +2371,14 @@
       </c>
       <c r="AD17" s="9">
         <f t="shared" si="10"/>
-        <v>170082</v>
+        <v>170084</v>
       </c>
       <c r="AE17" s="22">
-        <v>769911</v>
+        <v>769913</v>
       </c>
       <c r="AF17" s="10">
         <f t="shared" si="11"/>
-        <v>0.90843669470166799</v>
+        <v>0.90843905455026008</v>
       </c>
       <c r="AG17" s="6">
         <v>284469</v>
@@ -2498,14 +2498,14 @@
       </c>
       <c r="T18" s="9">
         <f t="shared" si="6"/>
-        <v>11743</v>
+        <v>11744</v>
       </c>
       <c r="U18" s="22">
-        <v>61026</v>
+        <v>61027</v>
       </c>
       <c r="V18" s="10">
         <f t="shared" si="7"/>
-        <v>0.75567443069950591</v>
+        <v>0.75568681352700073</v>
       </c>
       <c r="W18" s="6">
         <v>83269</v>
@@ -2515,14 +2515,14 @@
       </c>
       <c r="Y18" s="9">
         <f t="shared" si="8"/>
-        <v>13395</v>
+        <v>13396</v>
       </c>
       <c r="Z18" s="22">
-        <v>63335</v>
+        <v>63336</v>
       </c>
       <c r="AA18" s="10">
         <f t="shared" si="9"/>
-        <v>0.76060718874971478</v>
+        <v>0.76061919802087208</v>
       </c>
       <c r="AB18" s="6">
         <v>219776</v>
@@ -2549,14 +2549,14 @@
       </c>
       <c r="AI18" s="9">
         <f t="shared" si="12"/>
-        <v>16162</v>
+        <v>16163</v>
       </c>
       <c r="AJ18" s="22">
-        <v>64271</v>
+        <v>64272</v>
       </c>
       <c r="AK18" s="10">
         <f t="shared" si="13"/>
-        <v>0.74167974519940916</v>
+        <v>0.74169128508124071</v>
       </c>
       <c r="AL18" s="6">
         <v>88999</v>
@@ -3591,14 +3591,14 @@
       </c>
       <c r="J25" s="9">
         <f t="shared" si="2"/>
-        <v>1315</v>
+        <v>1317</v>
       </c>
       <c r="K25" s="22">
-        <v>5486</v>
+        <v>5488</v>
       </c>
       <c r="L25" s="10">
         <f t="shared" si="3"/>
-        <v>0.72231731402238319</v>
+        <v>0.72258064516129028</v>
       </c>
       <c r="M25" s="6">
         <v>14696</v>
@@ -3608,14 +3608,14 @@
       </c>
       <c r="O25" s="9">
         <f t="shared" si="4"/>
-        <v>3221</v>
+        <v>3223</v>
       </c>
       <c r="P25" s="22">
-        <v>11742</v>
+        <v>11744</v>
       </c>
       <c r="Q25" s="10">
         <f t="shared" si="5"/>
-        <v>0.79899292324442028</v>
+        <v>0.799129014697877</v>
       </c>
       <c r="R25" s="6">
         <v>8161</v>
@@ -3625,14 +3625,14 @@
       </c>
       <c r="T25" s="9">
         <f t="shared" si="6"/>
-        <v>1601</v>
+        <v>1603</v>
       </c>
       <c r="U25" s="22">
-        <v>6010</v>
+        <v>6012</v>
       </c>
       <c r="V25" s="10">
         <f t="shared" si="7"/>
-        <v>0.73642935914716334</v>
+        <v>0.73667442715353515</v>
       </c>
       <c r="W25" s="6">
         <v>8403</v>
@@ -3642,14 +3642,14 @@
       </c>
       <c r="Y25" s="9">
         <f t="shared" si="8"/>
-        <v>1724</v>
+        <v>1726</v>
       </c>
       <c r="Z25" s="22">
-        <v>6241</v>
+        <v>6243</v>
       </c>
       <c r="AA25" s="10">
         <f t="shared" si="9"/>
-        <v>0.74271093657027254</v>
+        <v>0.74294894680471257</v>
       </c>
       <c r="AB25" s="6">
         <v>15398</v>
@@ -3659,14 +3659,14 @@
       </c>
       <c r="AD25" s="9">
         <f t="shared" si="10"/>
-        <v>3680</v>
+        <v>3682</v>
       </c>
       <c r="AE25" s="22">
-        <v>12357</v>
+        <v>12359</v>
       </c>
       <c r="AF25" s="10">
         <f t="shared" si="11"/>
-        <v>0.80250681906741139</v>
+        <v>0.80263670606572279</v>
       </c>
       <c r="AG25" s="6">
         <v>8752</v>
@@ -3676,14 +3676,14 @@
       </c>
       <c r="AI25" s="9">
         <f t="shared" si="12"/>
-        <v>1961</v>
+        <v>1962</v>
       </c>
       <c r="AJ25" s="22">
-        <v>6319</v>
+        <v>6320</v>
       </c>
       <c r="AK25" s="10">
         <f t="shared" si="13"/>
-        <v>0.72200639853747717</v>
+        <v>0.72212065813528337</v>
       </c>
       <c r="AL25" s="6">
         <v>8845</v>
@@ -3693,14 +3693,14 @@
       </c>
       <c r="AN25" s="9">
         <f t="shared" si="14"/>
-        <v>2106</v>
+        <v>2107</v>
       </c>
       <c r="AO25" s="22">
-        <v>6376</v>
+        <v>6377</v>
       </c>
       <c r="AP25" s="10">
         <f t="shared" si="15"/>
-        <v>0.72085924250989264</v>
+        <v>0.7209723007348785</v>
       </c>
       <c r="AQ25" s="6">
         <v>16327</v>
@@ -3803,14 +3803,14 @@
       </c>
       <c r="Y26" s="9">
         <f t="shared" si="8"/>
-        <v>8882</v>
+        <v>8883</v>
       </c>
       <c r="Z26" s="22">
-        <v>39491</v>
+        <v>39492</v>
       </c>
       <c r="AA26" s="10">
         <f t="shared" si="9"/>
-        <v>0.70790162406338508</v>
+        <v>0.70791954970781201</v>
       </c>
       <c r="AB26" s="6">
         <v>114563</v>
@@ -3820,14 +3820,14 @@
       </c>
       <c r="AD26" s="9">
         <f t="shared" si="10"/>
-        <v>28767</v>
+        <v>28768</v>
       </c>
       <c r="AE26" s="22">
-        <v>91595</v>
+        <v>91596</v>
       </c>
       <c r="AF26" s="10">
         <f t="shared" si="11"/>
-        <v>0.79951642327802175</v>
+        <v>0.79952515209971808</v>
       </c>
       <c r="AG26" s="6">
         <v>56208</v>
@@ -3981,14 +3981,14 @@
       </c>
       <c r="AD27" s="9">
         <f t="shared" si="10"/>
-        <v>64103</v>
+        <v>64104</v>
       </c>
       <c r="AE27" s="22">
-        <v>408371</v>
+        <v>408372</v>
       </c>
       <c r="AF27" s="10">
         <f t="shared" si="11"/>
-        <v>0.91997828300577622</v>
+        <v>0.91998053580600692</v>
       </c>
       <c r="AG27" s="6">
         <v>164959</v>
@@ -4413,14 +4413,14 @@
       </c>
       <c r="O30" s="9">
         <f t="shared" si="4"/>
-        <v>20870</v>
+        <v>20871</v>
       </c>
       <c r="P30" s="22">
-        <v>81246</v>
+        <v>81247</v>
       </c>
       <c r="Q30" s="10">
         <f t="shared" si="5"/>
-        <v>0.86447549024823633</v>
+        <v>0.86448613047040423</v>
       </c>
       <c r="R30" s="6">
         <v>36736</v>
@@ -4447,14 +4447,14 @@
       </c>
       <c r="Y30" s="9">
         <f t="shared" si="8"/>
-        <v>5036</v>
+        <v>5037</v>
       </c>
       <c r="Z30" s="22">
-        <v>30691</v>
+        <v>30692</v>
       </c>
       <c r="AA30" s="10">
         <f t="shared" si="9"/>
-        <v>0.821889561351829</v>
+        <v>0.82191634084944565</v>
       </c>
       <c r="AB30" s="6">
         <v>90937</v>
@@ -4574,14 +4574,14 @@
       </c>
       <c r="O31" s="9">
         <f t="shared" si="4"/>
-        <v>53551</v>
+        <v>53552</v>
       </c>
       <c r="P31" s="22">
-        <v>265708</v>
+        <v>265709</v>
       </c>
       <c r="Q31" s="10">
         <f t="shared" si="5"/>
-        <v>0.91513001549853623</v>
+        <v>0.91513345961770276</v>
       </c>
       <c r="R31" s="6">
         <v>95518</v>
@@ -4625,14 +4625,14 @@
       </c>
       <c r="AD31" s="9">
         <f t="shared" si="10"/>
-        <v>56143</v>
+        <v>56146</v>
       </c>
       <c r="AE31" s="22">
-        <v>261926</v>
+        <v>261929</v>
       </c>
       <c r="AF31" s="10">
         <f t="shared" si="11"/>
-        <v>0.91310183264598943</v>
+        <v>0.91311229096436153</v>
       </c>
       <c r="AG31" s="6">
         <v>99962</v>
@@ -4642,14 +4642,14 @@
       </c>
       <c r="AI31" s="9">
         <f t="shared" si="12"/>
-        <v>11513</v>
+        <v>11514</v>
       </c>
       <c r="AJ31" s="22">
-        <v>84146</v>
+        <v>84147</v>
       </c>
       <c r="AK31" s="10">
         <f t="shared" si="13"/>
-        <v>0.8417798763530141</v>
+        <v>0.84178988015445866</v>
       </c>
       <c r="AL31" s="6">
         <v>100963</v>
@@ -4676,14 +4676,14 @@
       </c>
       <c r="AS31" s="9">
         <f t="shared" si="16"/>
-        <v>72145</v>
+        <v>72146</v>
       </c>
       <c r="AT31" s="22">
-        <v>273903</v>
+        <v>273904</v>
       </c>
       <c r="AU31" s="10">
         <f t="shared" si="17"/>
-        <v>0.89825172417185639</v>
+        <v>0.8982550036237944</v>
       </c>
     </row>
     <row r="32" spans="1:47" x14ac:dyDescent="0.3">
@@ -4718,14 +4718,14 @@
       </c>
       <c r="J32" s="9">
         <f t="shared" si="2"/>
-        <v>8459</v>
+        <v>8460</v>
       </c>
       <c r="K32" s="22">
-        <v>204579</v>
+        <v>204580</v>
       </c>
       <c r="L32" s="10">
         <f t="shared" si="3"/>
-        <v>0.91047014633104284</v>
+        <v>0.91047459678854992</v>
       </c>
       <c r="M32" s="6">
         <v>682019</v>
@@ -4735,14 +4735,14 @@
       </c>
       <c r="O32" s="9">
         <f t="shared" si="4"/>
-        <v>94832</v>
+        <v>94835</v>
       </c>
       <c r="P32" s="22">
-        <v>656101</v>
+        <v>656104</v>
       </c>
       <c r="Q32" s="10">
         <f t="shared" si="5"/>
-        <v>0.96199812615191072</v>
+        <v>0.96200252485634563</v>
       </c>
       <c r="R32" s="6">
         <v>225967</v>
@@ -4786,14 +4786,14 @@
       </c>
       <c r="AD32" s="9">
         <f t="shared" si="10"/>
-        <v>100365</v>
+        <v>100367</v>
       </c>
       <c r="AE32" s="22">
-        <v>678199</v>
+        <v>678201</v>
       </c>
       <c r="AF32" s="10">
         <f t="shared" si="11"/>
-        <v>0.97042364162668537</v>
+        <v>0.9704265033933398</v>
       </c>
       <c r="AG32" s="6">
         <v>232401</v>
@@ -4837,14 +4837,14 @@
       </c>
       <c r="AS32" s="9">
         <f t="shared" si="16"/>
-        <v>118437</v>
+        <v>118440</v>
       </c>
       <c r="AT32" s="22">
-        <v>708221</v>
+        <v>708224</v>
       </c>
       <c r="AU32" s="10">
         <f t="shared" si="17"/>
-        <v>0.96578532164388642</v>
+        <v>0.9657894126775679</v>
       </c>
     </row>
     <row r="33" spans="1:47" x14ac:dyDescent="0.3">
@@ -5252,14 +5252,14 @@
       </c>
       <c r="Y35" s="9">
         <f t="shared" si="8"/>
-        <v>30175</v>
+        <v>30176</v>
       </c>
       <c r="Z35" s="22">
-        <v>313382</v>
+        <v>313383</v>
       </c>
       <c r="AA35" s="10">
         <f t="shared" si="9"/>
-        <v>0.91710197858411691</v>
+        <v>0.91710490505078879</v>
       </c>
       <c r="AB35" s="6">
         <v>1094504</v>
@@ -5269,14 +5269,14 @@
       </c>
       <c r="AD35" s="9">
         <f t="shared" si="10"/>
-        <v>211150</v>
+        <v>211151</v>
       </c>
       <c r="AE35" s="22">
-        <v>1042459</v>
+        <v>1042460</v>
       </c>
       <c r="AF35" s="10">
         <f t="shared" si="11"/>
-        <v>0.95244878045214998</v>
+        <v>0.95244969410801605</v>
       </c>
       <c r="AG35" s="6">
         <v>348478</v>
@@ -5286,14 +5286,14 @@
       </c>
       <c r="AI35" s="9">
         <f t="shared" si="12"/>
-        <v>36076</v>
+        <v>36078</v>
       </c>
       <c r="AJ35" s="22">
-        <v>316480</v>
+        <v>316482</v>
       </c>
       <c r="AK35" s="10">
         <f t="shared" si="13"/>
-        <v>0.90817784766900633</v>
+        <v>0.90818358691222978</v>
       </c>
       <c r="AL35" s="6">
         <v>352081</v>
@@ -5320,14 +5320,14 @@
       </c>
       <c r="AS35" s="9">
         <f t="shared" si="16"/>
-        <v>254042</v>
+        <v>254045</v>
       </c>
       <c r="AT35" s="22">
-        <v>1087101</v>
+        <v>1087104</v>
       </c>
       <c r="AU35" s="10">
         <f t="shared" si="17"/>
-        <v>0.94675168932011777</v>
+        <v>0.94675430200750188</v>
       </c>
     </row>
     <row r="36" spans="1:47" x14ac:dyDescent="0.3">
@@ -5345,14 +5345,14 @@
       </c>
       <c r="E36" s="9">
         <f t="shared" si="0"/>
-        <v>76415</v>
+        <v>76416</v>
       </c>
       <c r="F36" s="22">
-        <v>460734</v>
+        <v>460735</v>
       </c>
       <c r="G36" s="10">
         <f t="shared" si="1"/>
-        <v>0.9152316117972138</v>
+        <v>0.91523359826144646</v>
       </c>
       <c r="H36" s="6">
         <v>312358</v>
@@ -5362,14 +5362,14 @@
       </c>
       <c r="J36" s="9">
         <f t="shared" si="2"/>
-        <v>32466</v>
+        <v>32468</v>
       </c>
       <c r="K36" s="22">
-        <v>276709</v>
+        <v>276711</v>
       </c>
       <c r="L36" s="10">
         <f t="shared" si="3"/>
-        <v>0.88587133993686729</v>
+        <v>0.88587774284634935</v>
       </c>
       <c r="M36" s="6">
         <v>553919</v>
@@ -5379,14 +5379,14 @@
       </c>
       <c r="O36" s="9">
         <f t="shared" si="4"/>
-        <v>94063</v>
+        <v>94067</v>
       </c>
       <c r="P36" s="22">
-        <v>494803</v>
+        <v>494807</v>
       </c>
       <c r="Q36" s="10">
         <f t="shared" si="5"/>
-        <v>0.89327681484115906</v>
+        <v>0.89328403611358342</v>
       </c>
       <c r="R36" s="6">
         <v>318679</v>
@@ -5396,14 +5396,14 @@
       </c>
       <c r="T36" s="9">
         <f t="shared" si="6"/>
-        <v>35619</v>
+        <v>35620</v>
       </c>
       <c r="U36" s="22">
-        <v>284074</v>
+        <v>284075</v>
       </c>
       <c r="V36" s="10">
         <f t="shared" si="7"/>
-        <v>0.89141110647391264</v>
+        <v>0.89141424442777839</v>
       </c>
       <c r="W36" s="6">
         <v>324721</v>
@@ -5413,14 +5413,14 @@
       </c>
       <c r="Y36" s="9">
         <f t="shared" si="8"/>
-        <v>38964</v>
+        <v>38965</v>
       </c>
       <c r="Z36" s="22">
-        <v>289580</v>
+        <v>289581</v>
       </c>
       <c r="AA36" s="10">
         <f t="shared" si="9"/>
-        <v>0.89178094425676191</v>
+        <v>0.8917840238235285</v>
       </c>
       <c r="AB36" s="6">
         <v>556414</v>
@@ -5430,14 +5430,14 @@
       </c>
       <c r="AD36" s="9">
         <f t="shared" si="10"/>
-        <v>102239</v>
+        <v>102243</v>
       </c>
       <c r="AE36" s="22">
-        <v>499766</v>
+        <v>499770</v>
       </c>
       <c r="AF36" s="10">
         <f t="shared" si="11"/>
-        <v>0.89819091539752771</v>
+        <v>0.89819810428925229</v>
       </c>
       <c r="AG36" s="6">
         <v>333690</v>
@@ -5447,14 +5447,14 @@
       </c>
       <c r="AI36" s="9">
         <f t="shared" si="12"/>
-        <v>47433</v>
+        <v>47436</v>
       </c>
       <c r="AJ36" s="22">
-        <v>293792</v>
+        <v>293795</v>
       </c>
       <c r="AK36" s="10">
         <f t="shared" si="13"/>
-        <v>0.88043393568881301</v>
+        <v>0.88044292606910601</v>
       </c>
       <c r="AL36" s="6">
         <v>339216</v>
@@ -5464,14 +5464,14 @@
       </c>
       <c r="AN36" s="9">
         <f t="shared" si="14"/>
-        <v>52342</v>
+        <v>52344</v>
       </c>
       <c r="AO36" s="22">
-        <v>296778</v>
+        <v>296780</v>
       </c>
       <c r="AP36" s="10">
         <f t="shared" si="15"/>
-        <v>0.87489387293052212</v>
+        <v>0.87489976887882648</v>
       </c>
       <c r="AQ36" s="6">
         <v>590015</v>
@@ -5481,14 +5481,14 @@
       </c>
       <c r="AS36" s="9">
         <f t="shared" si="16"/>
-        <v>131211</v>
+        <v>131215</v>
       </c>
       <c r="AT36" s="22">
-        <v>521193</v>
+        <v>521197</v>
       </c>
       <c r="AU36" s="10">
         <f t="shared" si="17"/>
-        <v>0.88335550791081585</v>
+        <v>0.88336228739947287</v>
       </c>
     </row>
     <row r="37" spans="1:47" x14ac:dyDescent="0.3">
@@ -5964,14 +5964,14 @@
       </c>
       <c r="AS39" s="9">
         <f t="shared" si="16"/>
-        <v>50863</v>
+        <v>50864</v>
       </c>
       <c r="AT39" s="22">
-        <v>233367</v>
+        <v>233368</v>
       </c>
       <c r="AU39" s="10">
         <f t="shared" si="17"/>
-        <v>0.94956889010054479</v>
+        <v>0.94957295909440476</v>
       </c>
     </row>
     <row r="40" spans="1:47" x14ac:dyDescent="0.3">
@@ -6006,14 +6006,14 @@
       </c>
       <c r="J40" s="9">
         <f t="shared" si="2"/>
-        <v>35832</v>
+        <v>35840</v>
       </c>
       <c r="K40" s="22">
-        <v>381009</v>
+        <v>381017</v>
       </c>
       <c r="L40" s="10">
         <f t="shared" si="3"/>
-        <v>0.87210164665381817</v>
+        <v>0.87211995806686415</v>
       </c>
       <c r="M40" s="6">
         <v>700632</v>
@@ -6023,14 +6023,14 @@
       </c>
       <c r="O40" s="9">
         <f t="shared" si="4"/>
-        <v>101884</v>
+        <v>101901</v>
       </c>
       <c r="P40" s="22">
-        <v>625013</v>
+        <v>625030</v>
       </c>
       <c r="Q40" s="10">
         <f t="shared" si="5"/>
-        <v>0.89207030224140493</v>
+        <v>0.89209456604893866</v>
       </c>
       <c r="R40" s="6">
         <v>444591</v>
@@ -6040,14 +6040,14 @@
       </c>
       <c r="T40" s="9">
         <f t="shared" si="6"/>
-        <v>39773</v>
+        <v>39778</v>
       </c>
       <c r="U40" s="22">
-        <v>390976</v>
+        <v>390981</v>
       </c>
       <c r="V40" s="10">
         <f t="shared" si="7"/>
-        <v>0.8794060158662681</v>
+        <v>0.87941726215780347</v>
       </c>
       <c r="W40" s="6">
         <v>452148</v>
@@ -6057,14 +6057,14 @@
       </c>
       <c r="Y40" s="9">
         <f t="shared" si="8"/>
-        <v>43501</v>
+        <v>43505</v>
       </c>
       <c r="Z40" s="22">
-        <v>397650</v>
+        <v>397654</v>
       </c>
       <c r="AA40" s="10">
         <f t="shared" si="9"/>
-        <v>0.87946866955067815</v>
+        <v>0.87947751621150594</v>
       </c>
       <c r="AB40" s="6">
         <v>712131</v>
@@ -6074,14 +6074,14 @@
       </c>
       <c r="AD40" s="9">
         <f t="shared" si="10"/>
-        <v>112256</v>
+        <v>112273</v>
       </c>
       <c r="AE40" s="22">
-        <v>635569</v>
+        <v>635586</v>
       </c>
       <c r="AF40" s="10">
         <f t="shared" si="11"/>
-        <v>0.89248888196132448</v>
+        <v>0.89251275397363683</v>
       </c>
       <c r="AG40" s="6">
         <v>463481</v>
@@ -6091,14 +6091,14 @@
       </c>
       <c r="AI40" s="9">
         <f t="shared" si="12"/>
-        <v>52794</v>
+        <v>52802</v>
       </c>
       <c r="AJ40" s="22">
-        <v>402873</v>
+        <v>402881</v>
       </c>
       <c r="AK40" s="10">
         <f t="shared" si="13"/>
-        <v>0.86923304299421122</v>
+        <v>0.86925030368019396</v>
       </c>
       <c r="AL40" s="6">
         <v>472374</v>
@@ -6108,14 +6108,14 @@
       </c>
       <c r="AN40" s="9">
         <f t="shared" si="14"/>
-        <v>58021</v>
+        <v>58029</v>
       </c>
       <c r="AO40" s="22">
-        <v>408077</v>
+        <v>408085</v>
       </c>
       <c r="AP40" s="10">
         <f t="shared" si="15"/>
-        <v>0.86388539589393154</v>
+        <v>0.86390233162705821</v>
       </c>
       <c r="AQ40" s="6">
         <v>750910</v>
@@ -6125,14 +6125,14 @@
       </c>
       <c r="AS40" s="9">
         <f t="shared" si="16"/>
-        <v>139006</v>
+        <v>139021</v>
       </c>
       <c r="AT40" s="22">
-        <v>659164</v>
+        <v>659179</v>
       </c>
       <c r="AU40" s="10">
         <f t="shared" si="17"/>
-        <v>0.87782024476967946</v>
+        <v>0.87784022053242061</v>
       </c>
     </row>
     <row r="41" spans="1:47" x14ac:dyDescent="0.3">
@@ -6506,14 +6506,14 @@
       </c>
       <c r="O43" s="9">
         <f t="shared" si="4"/>
-        <v>35000</v>
+        <v>35001</v>
       </c>
       <c r="P43" s="22">
-        <v>203714</v>
+        <v>203715</v>
       </c>
       <c r="Q43" s="10">
         <f t="shared" si="5"/>
-        <v>0.86725558228144495</v>
+        <v>0.86725983950275654</v>
       </c>
       <c r="R43" s="6">
         <v>144948</v>
@@ -6523,14 +6523,14 @@
       </c>
       <c r="T43" s="9">
         <f t="shared" si="6"/>
-        <v>15658</v>
+        <v>15659</v>
       </c>
       <c r="U43" s="22">
-        <v>124551</v>
+        <v>124552</v>
       </c>
       <c r="V43" s="10">
         <f t="shared" si="7"/>
-        <v>0.85928056958357479</v>
+        <v>0.85928746860943239</v>
       </c>
       <c r="W43" s="6">
         <v>148881</v>
@@ -6650,14 +6650,14 @@
       </c>
       <c r="J44" s="9">
         <f t="shared" si="2"/>
-        <v>10404</v>
+        <v>10406</v>
       </c>
       <c r="K44" s="22">
-        <v>110522</v>
+        <v>110524</v>
       </c>
       <c r="L44" s="10">
         <f t="shared" si="3"/>
-        <v>0.85277346974992863</v>
+        <v>0.85278890149147779</v>
       </c>
       <c r="M44" s="6">
         <v>216950</v>
@@ -6667,14 +6667,14 @@
       </c>
       <c r="O44" s="9">
         <f t="shared" si="4"/>
-        <v>33749</v>
+        <v>33751</v>
       </c>
       <c r="P44" s="22">
-        <v>192107</v>
+        <v>192109</v>
       </c>
       <c r="Q44" s="10">
         <f t="shared" si="5"/>
-        <v>0.88548974418068682</v>
+        <v>0.88549896289467622</v>
       </c>
       <c r="R44" s="6">
         <v>129192</v>
@@ -6684,14 +6684,14 @@
       </c>
       <c r="T44" s="9">
         <f t="shared" si="6"/>
-        <v>11753</v>
+        <v>11754</v>
       </c>
       <c r="U44" s="22">
-        <v>113813</v>
+        <v>113814</v>
       </c>
       <c r="V44" s="10">
         <f t="shared" si="7"/>
-        <v>0.88096012136974422</v>
+        <v>0.88096786178710751</v>
       </c>
       <c r="W44" s="6">
         <v>132744</v>
@@ -6701,14 +6701,14 @@
       </c>
       <c r="Y44" s="9">
         <f t="shared" si="8"/>
-        <v>13178</v>
+        <v>13179</v>
       </c>
       <c r="Z44" s="22">
-        <v>116682</v>
+        <v>116683</v>
       </c>
       <c r="AA44" s="10">
         <f t="shared" si="9"/>
-        <v>0.87900018079913211</v>
+        <v>0.87900771409630563</v>
       </c>
       <c r="AB44" s="6">
         <v>215764</v>
@@ -6718,14 +6718,14 @@
       </c>
       <c r="AD44" s="9">
         <f t="shared" si="10"/>
-        <v>36156</v>
+        <v>36157</v>
       </c>
       <c r="AE44" s="22">
-        <v>193270</v>
+        <v>193271</v>
       </c>
       <c r="AF44" s="10">
         <f t="shared" si="11"/>
-        <v>0.89574720527984275</v>
+        <v>0.89575183997330421</v>
       </c>
       <c r="AG44" s="6">
         <v>134716</v>
@@ -6735,14 +6735,14 @@
       </c>
       <c r="AI44" s="9">
         <f t="shared" si="12"/>
-        <v>15808</v>
+        <v>15809</v>
       </c>
       <c r="AJ44" s="22">
-        <v>118326</v>
+        <v>118327</v>
       </c>
       <c r="AK44" s="10">
         <f t="shared" si="13"/>
-        <v>0.87833664895038455</v>
+        <v>0.8783440719736334</v>
       </c>
       <c r="AL44" s="6">
         <v>136843</v>
@@ -6752,14 +6752,14 @@
       </c>
       <c r="AN44" s="9">
         <f t="shared" si="14"/>
-        <v>17427</v>
+        <v>17428</v>
       </c>
       <c r="AO44" s="22">
-        <v>119596</v>
+        <v>119597</v>
       </c>
       <c r="AP44" s="10">
         <f t="shared" si="15"/>
-        <v>0.87396505484387221</v>
+        <v>0.87397236248839916</v>
       </c>
       <c r="AQ44" s="6">
         <v>226630</v>
@@ -6769,14 +6769,14 @@
       </c>
       <c r="AS44" s="9">
         <f t="shared" si="16"/>
-        <v>45593</v>
+        <v>45594</v>
       </c>
       <c r="AT44" s="22">
-        <v>201462</v>
+        <v>201463</v>
       </c>
       <c r="AU44" s="10">
         <f t="shared" si="17"/>
-        <v>0.8889467413846357</v>
+        <v>0.88895115386312495</v>
       </c>
     </row>
     <row r="45" spans="1:47" x14ac:dyDescent="0.3">
@@ -7082,10 +7082,10 @@
       </c>
     </row>
     <row r="47" spans="1:47" s="3" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="26" t="s">
+      <c r="A47" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="B47" s="26"/>
+      <c r="B47" s="29"/>
       <c r="C47" s="13">
         <f>SUM(C9:C46)</f>
         <v>6783589</v>
@@ -7096,15 +7096,15 @@
       </c>
       <c r="E47" s="11">
         <f>F47-D47</f>
-        <v>989605</v>
+        <v>989606</v>
       </c>
       <c r="F47" s="13">
         <f>SUM(F9:F46)</f>
-        <v>6283608</v>
+        <v>6283609</v>
       </c>
       <c r="G47" s="12">
         <f>F47/C47</f>
-        <v>0.92629550522592097</v>
+        <v>0.92629565264051228</v>
       </c>
       <c r="H47" s="13">
         <f>SUM(H9:H46)</f>
@@ -7116,15 +7116,15 @@
       </c>
       <c r="J47" s="11">
         <f t="shared" si="2"/>
-        <v>240284</v>
+        <v>240299</v>
       </c>
       <c r="K47" s="13">
         <f>SUM(K9:K46)</f>
-        <v>2669810</v>
+        <v>2669825</v>
       </c>
       <c r="L47" s="12">
         <f t="shared" si="3"/>
-        <v>0.84822761822338633</v>
+        <v>0.8482323838862138</v>
       </c>
       <c r="M47" s="13">
         <f>SUM(M9:M46)</f>
@@ -7136,15 +7136,15 @@
       </c>
       <c r="O47" s="11">
         <f t="shared" si="4"/>
-        <v>1297193</v>
+        <v>1297228</v>
       </c>
       <c r="P47" s="13">
         <f>SUM(P9:P46)</f>
-        <v>7192237</v>
+        <v>7192272</v>
       </c>
       <c r="Q47" s="12">
         <f t="shared" si="5"/>
-        <v>0.91772400717260871</v>
+        <v>0.91772847314616479</v>
       </c>
       <c r="R47" s="13">
         <f>SUM(R9:R46)</f>
@@ -7156,15 +7156,15 @@
       </c>
       <c r="T47" s="11">
         <f t="shared" si="6"/>
-        <v>273676</v>
+        <v>273688</v>
       </c>
       <c r="U47" s="13">
         <f>SUM(U9:U46)</f>
-        <v>2762809</v>
+        <v>2762821</v>
       </c>
       <c r="V47" s="12">
         <f t="shared" si="7"/>
-        <v>0.87431190250827462</v>
+        <v>0.87431569999946201</v>
       </c>
       <c r="W47" s="13">
         <f>SUM(W9:W46)</f>
@@ -7176,15 +7176,15 @@
       </c>
       <c r="Y47" s="11">
         <f t="shared" si="8"/>
-        <v>309669</v>
+        <v>309682</v>
       </c>
       <c r="Z47" s="13">
         <f>SUM(Z9:Z46)</f>
-        <v>2821223</v>
+        <v>2821236</v>
       </c>
       <c r="AA47" s="12">
         <f t="shared" si="9"/>
-        <v>0.87846313175220392</v>
+        <v>0.87846717964941479</v>
       </c>
       <c r="AB47" s="13">
         <f>SUM(AB9:AB46)</f>
@@ -7196,15 +7196,15 @@
       </c>
       <c r="AD47" s="11">
         <f t="shared" si="10"/>
-        <v>1416883</v>
+        <v>1416920</v>
       </c>
       <c r="AE47" s="13">
         <f>SUM(AE9:AE46)</f>
-        <v>7335753</v>
+        <v>7335790</v>
       </c>
       <c r="AF47" s="12">
         <f t="shared" si="11"/>
-        <v>0.92031954831564311</v>
+        <v>0.92032419021447576</v>
       </c>
       <c r="AG47" s="13">
         <f>SUM(AG9:AG46)</f>
@@ -7216,15 +7216,15 @@
       </c>
       <c r="AI47" s="11">
         <f t="shared" si="12"/>
-        <v>368876</v>
+        <v>368895</v>
       </c>
       <c r="AJ47" s="13">
         <f>SUM(AJ9:AJ46)</f>
-        <v>2853807</v>
+        <v>2853826</v>
       </c>
       <c r="AK47" s="12">
         <f t="shared" si="13"/>
-        <v>0.86670936728974346</v>
+        <v>0.86671513764421326</v>
       </c>
       <c r="AL47" s="13">
         <f>SUM(AL9:AL46)</f>
@@ -7236,15 +7236,15 @@
       </c>
       <c r="AN47" s="11">
         <f t="shared" si="14"/>
-        <v>405332</v>
+        <v>405345</v>
       </c>
       <c r="AO47" s="13">
         <f>SUM(AO9:AO46)</f>
-        <v>2878507</v>
+        <v>2878520</v>
       </c>
       <c r="AP47" s="12">
         <f t="shared" si="15"/>
-        <v>0.8610782222674257</v>
+        <v>0.86108211109482458</v>
       </c>
       <c r="AQ47" s="13">
         <f>SUM(AQ9:AQ46)</f>
@@ -7256,15 +7256,15 @@
       </c>
       <c r="AS47" s="11">
         <f t="shared" si="16"/>
-        <v>1763045</v>
+        <v>1763082</v>
       </c>
       <c r="AT47" s="13">
         <f>SUM(AT9:AT46)</f>
-        <v>7684748</v>
+        <v>7684785</v>
       </c>
       <c r="AU47" s="12">
         <f t="shared" si="17"/>
-        <v>0.90883178113335805</v>
+        <v>0.90883615691456809</v>
       </c>
     </row>
     <row r="48" spans="1:47" x14ac:dyDescent="0.3">
@@ -7383,22 +7383,17 @@
       <c r="AT55" s="4"/>
     </row>
     <row r="56" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A56" s="27" t="s">
+      <c r="A56" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="B56" s="27"/>
-      <c r="C56" s="27"/>
-      <c r="D56" s="27"/>
-      <c r="E56" s="27"/>
+      <c r="B56" s="30"/>
+      <c r="C56" s="30"/>
+      <c r="D56" s="30"/>
+      <c r="E56" s="30"/>
       <c r="F56" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:G7"/>
     <mergeCell ref="AQ7:AU7"/>
     <mergeCell ref="A47:B47"/>
     <mergeCell ref="A56:E56"/>
@@ -7409,6 +7404,11 @@
     <mergeCell ref="AG7:AK7"/>
     <mergeCell ref="AL7:AP7"/>
     <mergeCell ref="H7:L7"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:G7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>